<commit_message>
add and update examples
</commit_message>
<xml_diff>
--- a/dev/lci-case-study-fertilizer_n2o_timing.xlsx
+++ b/dev/lci-case-study-fertilizer_n2o_timing.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T15"/>
+  <dimension ref="A1:DO19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -428,6 +428,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -679,7 +680,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>[0.1,0.1,0.1,0.1,0.1,0.1,0.1,0.1,0.1,0.1]</t>
+          <t>[0.16,0.14,0.12,0.11,0.1,0.1,0.09,0.08,0.06,0.04]</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -689,7 +690,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>Ammonia supply split across 10 biennial applications over 20 years.</t>
+          <t>Fertilizer dosing is front-loaded, then reduced as soil fertility and yield response stabilize.</t>
         </is>
       </c>
     </row>
@@ -738,7 +739,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>[0.1,0.1,0.1,0.1,0.1,0.1,0.1,0.1,0.1,0.1]</t>
+          <t>[0.14,0.13,0.12,0.11,0.1,0.1,0.1,0.09,0.07,0.04]</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -748,7 +749,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>Pumping and handling repeated every two years with fertilizer spreading.</t>
+          <t>Electricity for handling and application follows the fertilization campaign schedule.</t>
         </is>
       </c>
     </row>
@@ -792,7 +793,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>[0.008,0.016,0.026,0.034,0.04,0.034,0.051,0.034,0.06,0.034,0.066,0.034,0.066,0.034,0.066,0.034,0.066,0.034,0.066,0.034,0.058,0.018,0.04,0.026,0.015,0.006]</t>
+          <t>[0.114695,0.09319,0.086022,0.071685,0.064516,0.057348,0.053763,0.050179,0.046595,0.043011,0.039427,0.035842,0.032975,0.030108,0.02724,0.024373,0.021505,0.019355,0.017204,0.015054,0.012903,0.01147,0.010036,0.008602,0.007168,0.005734]</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -802,7 +803,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>N2O pulses follow each biennial fertilizer event and extend to year +28.</t>
+          <t>N2O peaks shortly after each application with a decaying multi-year soil emission tail.</t>
         </is>
       </c>
     </row>
@@ -846,7 +847,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>[0.055,0.025,0.068,0.032,0.068,0.032,0.068,0.032,0.068,0.032,0.068,0.032,0.068,0.032,0.068,0.032,0.068,0.032,0.068,0.032,0.013,0.007]</t>
+          <t>[0.153846,0.108597,0.090498,0.076923,0.067873,0.058824,0.054299,0.049774,0.045249,0.040724,0.037104,0.033484,0.029864,0.027149,0.024434,0.021719,0.019005,0.01629,0.01448,0.011765,0.009955,0.008144]</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -856,7 +857,233 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>NH3 volatilization follows each biennial application with short lag.</t>
+          <t>NH3 volatilization is strongest near application windows and declines quickly afterward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>market for diesel, low-sulfur</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Europe without Switzerland</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>kilogram</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>technosphere</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>diesel, low-sulfur</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>6</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>[0,2,4,6,8,10,12,14,16,18]</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>[0.14,0.13,0.12,0.11,0.1,0.1,0.1,0.09,0.07,0.04]</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>port</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Field machinery and transport diesel aligned with each fertilization operation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>market for tap water</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>24</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Europe without Switzerland</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>kilogram</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>technosphere</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>tap water</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>6</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>[0,2,4,6,8,10,12,14,16,18]</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>[0.14,0.13,0.12,0.11,0.1,0.1,0.1,0.09,0.07,0.04]</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>port</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Water used for fertilizer dilution and sprayer cleaning after field applications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Carbon dioxide, fossil</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>air::non-urban air or from high stacks</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>kilogram</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>biosphere</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>6</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>[0,2,4,6,8,10,12,14,16,18]</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>[0.14,0.13,0.12,0.11,0.1,0.1,0.1,0.09,0.07,0.04]</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>port</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Direct fossil CO2 from tractor operation tied to the fertilization schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Methane, fossil</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>air::non-urban air or from high stacks</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>kilogram</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>biosphere</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>6</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>21</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>[0,2,4,6,8,10,12,14,16,18,21]</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>[0.17,0.15,0.13,0.11,0.1,0.09,0.08,0.07,0.05,0.03,0.02]</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>port</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Fuel supply-chain methane associated with repeated machinery fuel demand.</t>
         </is>
       </c>
     </row>

</xml_diff>